<commit_message>
add more item on part list and receipts
</commit_message>
<xml_diff>
--- a/docs/part list.xlsx
+++ b/docs/part list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\pressure-sensing-cushion\resource\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\pressure-sensing-cushion\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98176010-613F-457A-8828-575E30FAB6FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB42CC1-77B3-4193-9904-2901945BE1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{039EFAA4-C4D2-4F31-ABF8-5ECCF156DD30}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{039EFAA4-C4D2-4F31-ABF8-5ECCF156DD30}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="5">
+  <futureMetadata name="XLRICHVALUE" count="9">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -79,8 +79,36 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="7"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="5">
+  <valueMetadata count="9">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -95,13 +123,25 @@
     </bk>
     <bk>
       <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+    <bk>
+      <rc t="1" v="7"/>
+    </bk>
+    <bk>
+      <rc t="1" v="8"/>
     </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Quantity</t>
   </si>
@@ -168,6 +208,9 @@
   </si>
   <si>
     <t>terminal for FSR</t>
+  </si>
+  <si>
+    <t>Receipt</t>
   </si>
 </sst>
 </file>
@@ -314,7 +357,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -333,6 +376,22 @@
   </rv>
   <rv s="0">
     <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>8</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -354,6 +413,10 @@
   <rel r:id="rId3"/>
   <rel r:id="rId4"/>
   <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
 </richValueRels>
 </file>
 
@@ -683,7 +746,8 @@
     <col min="4" max="4" width="68.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="32.28515625" style="1" customWidth="1"/>
     <col min="6" max="6" width="32" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="7" width="48.5703125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="5" customFormat="1" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -705,6 +769,9 @@
       <c r="F1" s="5" t="s">
         <v>0</v>
       </c>
+      <c r="G1" s="5" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="2" spans="1:9" ht="180" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -725,13 +792,16 @@
       <c r="F2" s="3">
         <v>4</v>
       </c>
+      <c r="G2" s="1" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" ht="284.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="e" vm="2">
+      <c r="B3" s="1" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
       <c r="C3" s="7" t="s">
@@ -745,13 +815,16 @@
       </c>
       <c r="F3" s="3">
         <v>1</v>
+      </c>
+      <c r="G3" s="1" t="e" vm="4">
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="278.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="1" t="e" vm="3">
+      <c r="B4" s="1" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
       <c r="C4" s="7" t="s">
@@ -765,13 +838,16 @@
       </c>
       <c r="F4" s="3">
         <v>2</v>
+      </c>
+      <c r="G4" s="1" t="e" vm="6">
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="320.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="1" t="e" vm="4">
+      <c r="B5" s="1" t="e" vm="7">
         <v>#VALUE!</v>
       </c>
       <c r="D5" s="8" t="s">
@@ -782,7 +858,7 @@
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="1" t="e" vm="5">
+      <c r="B6" s="1" t="e" vm="8">
         <v>#VALUE!</v>
       </c>
       <c r="C6" s="7" t="s">
@@ -796,6 +872,9 @@
       </c>
       <c r="F6" s="3">
         <v>4</v>
+      </c>
+      <c r="G6" s="1" t="e" vm="9">
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="195" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>